<commit_message>
feat(acompanhamento): transforma central em planilhas vivas editaveis
</commit_message>
<xml_diff>
--- a/fontes/acompanhamento/MKTG 2026.xlsx
+++ b/fontes/acompanhamento/MKTG 2026.xlsx
@@ -1,29 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marketing\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marketing\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985BEEBE-2662-4DD2-9DEB-80893BC32262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{BDFE9EE2-B36C-4ADD-964A-045A9F23A91A}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Planejamento" sheetId="1" r:id="rId1"/>
-    <sheet name="PODCAST" sheetId="10" r:id="rId2"/>
-    <sheet name="RECEITA" sheetId="3" r:id="rId3"/>
-    <sheet name="COPA" sheetId="13" r:id="rId4"/>
-    <sheet name="CONV FORNEC" sheetId="11" r:id="rId5"/>
-    <sheet name="PENDÊNCIAS" sheetId="4" r:id="rId6"/>
-    <sheet name="FIPAN" sheetId="5" r:id="rId7"/>
-    <sheet name="ANUGA" sheetId="6" r:id="rId8"/>
-    <sheet name="FISPAL" sheetId="7" r:id="rId9"/>
-    <sheet name="CONV VENDAS" sheetId="8" r:id="rId10"/>
-    <sheet name="CARTÃO" sheetId="9" r:id="rId11"/>
+    <sheet name="RECEITA" sheetId="3" r:id="rId2"/>
+    <sheet name="PENDÊNCIAS" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="140">
   <si>
     <t>Programação</t>
   </si>
@@ -465,208 +456,25 @@
     <t>HAVER</t>
   </si>
   <si>
-    <t>ESPAÇO</t>
-  </si>
-  <si>
-    <t>MONTAGEM</t>
-  </si>
-  <si>
-    <t>AUDIO E VIDEO</t>
-  </si>
-  <si>
-    <t>MONTAGEM STAND</t>
-  </si>
-  <si>
-    <t>SHOW STAND UP</t>
-  </si>
-  <si>
-    <t>GERADOR</t>
-  </si>
-  <si>
-    <t>BARTENDER</t>
-  </si>
-  <si>
-    <t>RODA DE SAMBA</t>
-  </si>
-  <si>
-    <t>FREEZER</t>
-  </si>
-  <si>
-    <t>MC</t>
-  </si>
-  <si>
-    <t>ILUMINAÇÃO</t>
-  </si>
-  <si>
-    <t>BRINDES</t>
-  </si>
-  <si>
-    <t>DIVERSOS</t>
-  </si>
-  <si>
-    <t>PAGO</t>
-  </si>
-  <si>
-    <t>INVESTIMENTO</t>
-  </si>
-  <si>
-    <t>ESTUDIO</t>
-  </si>
-  <si>
-    <t>PRODUTOS PMG</t>
-  </si>
-  <si>
-    <t>PALESTRANTE</t>
-  </si>
-  <si>
-    <t>HOMENAGEM</t>
-  </si>
-  <si>
-    <t>TENDA</t>
-  </si>
-  <si>
-    <t>CHINELOS</t>
-  </si>
-  <si>
-    <t>STAFF</t>
-  </si>
-  <si>
-    <t>AGUA / ENERGIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FREEZER / FORNO </t>
-  </si>
-  <si>
-    <t>CREDENCIAIS</t>
-  </si>
-  <si>
-    <t>POLTRONAS</t>
-  </si>
-  <si>
-    <t>CAMISETAS</t>
-  </si>
-  <si>
     <t>SEARA</t>
   </si>
   <si>
-    <t>LOCAÇÃO ESPAÇO + BUFFET</t>
-  </si>
-  <si>
-    <t>FALTA PAGAR</t>
-  </si>
-  <si>
     <t>PREDILECTA</t>
   </si>
   <si>
     <t>TOZZY</t>
   </si>
   <si>
-    <t>NITA</t>
-  </si>
-  <si>
-    <t>DESCARTÁVEIS</t>
-  </si>
-  <si>
-    <t>FOLDER</t>
-  </si>
-  <si>
-    <t>ENERGIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGUA  </t>
-  </si>
-  <si>
-    <t>AUDIO / SOM</t>
-  </si>
-  <si>
-    <t>FREE LANCE</t>
-  </si>
-  <si>
-    <t>CAMISA</t>
-  </si>
-  <si>
-    <t>BONE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOLA </t>
-  </si>
-  <si>
-    <t>MOCHILA</t>
-  </si>
-  <si>
     <t>DAUPHINE / FARM FRITES</t>
   </si>
   <si>
-    <t>MICROF</t>
-  </si>
-  <si>
-    <t>TRIPÉ</t>
-  </si>
-  <si>
-    <t>SMARTPHONE</t>
-  </si>
-  <si>
-    <t>KIT ILUMIN</t>
-  </si>
-  <si>
-    <t>ENERGIA/EXTI/AGUA</t>
-  </si>
-  <si>
-    <t>LOCAÇÃO FREEZER</t>
-  </si>
-  <si>
-    <t>SEGURO</t>
-  </si>
-  <si>
-    <t>CAMISAS</t>
-  </si>
-  <si>
-    <t>TABELA</t>
-  </si>
-  <si>
-    <t>LED</t>
-  </si>
-  <si>
-    <t>MUSICO</t>
-  </si>
-  <si>
-    <t>FREE LANCER</t>
-  </si>
-  <si>
-    <t>PEDIDOS</t>
-  </si>
-  <si>
-    <t>FORNO E FREEZER</t>
-  </si>
-  <si>
     <t>SIMPLOT</t>
-  </si>
-  <si>
-    <t>ML</t>
-  </si>
-  <si>
-    <t>Ffolder</t>
-  </si>
-  <si>
-    <t>PED PMG</t>
-  </si>
-  <si>
-    <t>PROD LIMP</t>
-  </si>
-  <si>
-    <t>MAGA LU</t>
-  </si>
-  <si>
-    <t>HONORARIOS</t>
-  </si>
-  <si>
-    <t>LONAS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
@@ -854,7 +662,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1266,32 +1074,6 @@
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1307,7 +1089,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1401,13 +1183,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1502,13 +1278,13 @@
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
-    <cellStyle name="Moeda 2" xfId="6" xr:uid="{CC9914C3-D3F1-4BEB-9804-616F28578787}"/>
-    <cellStyle name="Moeda 3" xfId="5" xr:uid="{E33311B7-0C7B-4BB1-B1A6-2768EFD612C6}"/>
+    <cellStyle name="Moeda 2" xfId="6"/>
+    <cellStyle name="Moeda 3" xfId="5"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{5C74F0C3-0677-4455-940C-EC168EB6DCC7}"/>
-    <cellStyle name="Normal 3" xfId="3" xr:uid="{C5684436-E622-4A66-92C8-25FB434FCF1D}"/>
-    <cellStyle name="Porcentagem 2" xfId="7" xr:uid="{381658A8-8B50-40CC-9E09-4FD0A22A1F75}"/>
-    <cellStyle name="WinCalendar_BlankCells_39" xfId="4" xr:uid="{92FCF2A0-5BE9-40B0-AE3D-005302B4E902}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 3" xfId="3"/>
+    <cellStyle name="Porcentagem 2" xfId="7"/>
+    <cellStyle name="WinCalendar_BlankCells_39" xfId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1819,47 +1595,47 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21A756C2-3F57-4424-9C8A-4439FCB7BE9B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.33203125" customWidth="1"/>
-    <col min="14" max="15" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" customWidth="1"/>
+    <col min="14" max="15" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="61" t="s">
+    <row r="1" spans="1:17" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="55" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="63"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="57"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1912,7 +1688,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>16</v>
       </c>
@@ -1952,7 +1728,7 @@
         <v>32667.48</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>17</v>
       </c>
@@ -1986,11 +1762,11 @@
       </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="8">
-        <f>SUM(B4:L4)</f>
+        <f t="shared" ref="Q4:Q11" si="0">SUM(B4:L4)</f>
         <v>21221.9</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
@@ -2030,15 +1806,15 @@
         <v>260869.18</v>
       </c>
       <c r="Q5" s="8">
-        <f>SUM(B5:L5)</f>
+        <f t="shared" si="0"/>
         <v>34766.729999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="60">
+      <c r="B6" s="54">
         <v>57135</v>
       </c>
       <c r="C6" s="4">
@@ -2049,7 +1825,7 @@
         <v>2639.4</v>
       </c>
       <c r="F6" s="4"/>
-      <c r="G6" s="54">
+      <c r="G6" s="53">
         <v>239873.27</v>
       </c>
       <c r="H6" s="4"/>
@@ -2074,11 +1850,11 @@
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="8">
-        <f>SUM(B6:L6)</f>
+        <f t="shared" si="0"/>
         <v>330642.67</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
@@ -2116,11 +1892,11 @@
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="8">
-        <f>SUM(B7:L7)</f>
+        <f t="shared" si="0"/>
         <v>61451.729999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
@@ -2158,11 +1934,11 @@
       </c>
       <c r="P8" s="4"/>
       <c r="Q8" s="8">
-        <f>SUM(B8:L8)</f>
+        <f t="shared" si="0"/>
         <v>845751.37000000011</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -2198,11 +1974,11 @@
       </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="8">
-        <f>SUM(B9:L9)</f>
+        <f t="shared" si="0"/>
         <v>519535.56</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
@@ -2242,11 +2018,11 @@
       </c>
       <c r="P10" s="4"/>
       <c r="Q10" s="8">
-        <f>SUM(B10:L10)</f>
+        <f t="shared" si="0"/>
         <v>55124.75</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
@@ -2284,11 +2060,11 @@
       </c>
       <c r="P11" s="4"/>
       <c r="Q11" s="8">
-        <f>SUM(B11:L11)</f>
+        <f t="shared" si="0"/>
         <v>65390</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>25</v>
       </c>
@@ -2328,7 +2104,7 @@
         <v>30434</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>26</v>
       </c>
@@ -2368,7 +2144,7 @@
         <v>11390</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>27</v>
       </c>
@@ -2410,7 +2186,7 @@
         <v>23390</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
         <v>28</v>
       </c>
@@ -2423,7 +2199,7 @@
         <v>15000</v>
       </c>
       <c r="D15" s="26">
-        <f t="shared" ref="D15:P15" si="0">SUM(D3:D14)</f>
+        <f t="shared" ref="D15:P15" si="1">SUM(D3:D14)</f>
         <v>32000</v>
       </c>
       <c r="E15" s="26">
@@ -2431,19 +2207,19 @@
         <v>31679.4</v>
       </c>
       <c r="F15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>38200</v>
       </c>
       <c r="G15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1596273.83</v>
       </c>
       <c r="H15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24000</v>
       </c>
       <c r="I15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>21000</v>
       </c>
       <c r="J15" s="26">
@@ -2451,11 +2227,11 @@
         <v>18000</v>
       </c>
       <c r="K15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>29000</v>
       </c>
       <c r="L15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>131333.19</v>
       </c>
       <c r="M15" s="26">
@@ -2463,15 +2239,15 @@
         <v>79248</v>
       </c>
       <c r="N15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>22280</v>
       </c>
       <c r="O15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>75730.080000000002</v>
       </c>
       <c r="P15" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>420869.18</v>
       </c>
       <c r="Q15" s="27">
@@ -2479,12 +2255,12 @@
         <v>2610377.6800000002</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="G18" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="29"/>
     </row>
   </sheetData>
@@ -2496,620 +2272,51 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BCB66C8-E58D-4C6C-911D-33DEF5A87799}">
-  <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:R79"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" customWidth="1"/>
-    <col min="3" max="3" width="36.5546875" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" style="9" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" style="10" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" customWidth="1"/>
+    <col min="11" max="11" width="17.42578125" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" customWidth="1"/>
+    <col min="13" max="17" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="22.140625" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="B1" s="4">
-        <v>15500</v>
-      </c>
-      <c r="C1" s="14"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="4">
-        <v>15500</v>
-      </c>
-      <c r="C2" s="14"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="B3" s="4">
-        <v>32655</v>
-      </c>
-      <c r="C3" s="14"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
-      <c r="B4" s="4">
-        <v>32655</v>
-      </c>
-      <c r="C4" s="14"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="B5" s="4">
-        <v>7500</v>
-      </c>
-      <c r="C5" s="14"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="B6" s="4">
-        <v>5550</v>
-      </c>
-      <c r="C6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="B7" s="4">
-        <v>4100</v>
-      </c>
-      <c r="C7" s="14"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="B8" s="4">
-        <v>4500</v>
-      </c>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B9" s="4">
-        <v>44779</v>
-      </c>
-      <c r="C9" s="14"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="B10" s="4">
-        <v>13320</v>
-      </c>
-      <c r="C10" s="14"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="B11" s="4">
-        <v>5000</v>
-      </c>
-      <c r="C11" s="14"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="B12" s="4">
-        <v>5800</v>
-      </c>
-      <c r="C12" s="14"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="B13" s="4">
-        <v>17990.02</v>
-      </c>
-      <c r="C13" s="14"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B14" s="4">
-        <v>4341.26</v>
-      </c>
-      <c r="C14" s="14"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="B15" s="4">
-        <v>8401.9</v>
-      </c>
-      <c r="C15" s="14"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="B16" s="4">
-        <v>13000</v>
-      </c>
-      <c r="C16" s="14"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="B17" s="4">
-        <v>9024</v>
-      </c>
-      <c r="C17" s="14"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="B18" s="4">
-        <v>900</v>
-      </c>
-      <c r="C18" s="14"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="B19" s="4">
-        <v>4225</v>
-      </c>
-      <c r="C19" s="14"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20" s="4">
-        <v>3100</v>
-      </c>
-      <c r="C20" s="14"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="B21" s="4">
-        <v>2180</v>
-      </c>
-      <c r="C21" s="14"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="B22" s="4">
-        <v>2160</v>
-      </c>
-      <c r="C22" s="14"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="B23" s="4">
-        <v>1398</v>
-      </c>
-      <c r="C23" s="14"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="B24" s="4">
-        <v>7290</v>
-      </c>
-      <c r="C24" s="14"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="14"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="14"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="14"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="14"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="14"/>
-      <c r="B28" s="4">
-        <f>SUM(B1:B27)</f>
-        <v>260869.18</v>
-      </c>
-      <c r="C28" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F5BBF49-096D-4558-9D91-8159CDE69F32}">
-  <dimension ref="A2:D20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="27.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="53"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="53"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="53"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="55"/>
-      <c r="B5" s="56"/>
-      <c r="C5" s="57"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="53">
-        <v>46205</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="C6" s="4">
-        <v>2475.85</v>
-      </c>
-      <c r="D6" s="14">
-        <v>260.89999999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="53"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="14">
-        <v>314.7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="53"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="14">
-        <v>1528.95</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="53"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="14">
-        <v>406.9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="14">
-        <f>SUM(D6:D9)</f>
-        <v>2511.4500000000003</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="58"/>
-      <c r="B11" s="58" t="s">
-        <v>198</v>
-      </c>
-      <c r="C11" s="59">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14" t="s">
-        <v>198</v>
-      </c>
-      <c r="C12" s="4">
-        <v>279.51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="4"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="4"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="14"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="4"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="4"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="4"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="4"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2C7A858-FD8F-4999-94A7-F53BEA33FFC7}">
-  <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="4">
-        <v>10000</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" s="4">
-        <v>8000</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="4">
-        <v>10000</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="14"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="14"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="14"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="14"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="14"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="14"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
-      <c r="B10" s="4">
-        <f>SUM(B1:B9)</f>
-        <v>28000</v>
-      </c>
-      <c r="C10" s="14"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B11" s="10"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B12" s="10"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B13" s="10"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B14" s="10"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B15" s="10"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="B16" s="4">
-        <v>32000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="B18" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="B19" s="4">
-        <v>856.75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="B20" s="4">
-        <v>798.54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="B21" s="4">
-        <v>10553.44</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="B22" s="4">
-        <v>531.99</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="14"/>
-      <c r="B23" s="4"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
-      <c r="B24" s="4"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="4"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="14"/>
-      <c r="B27" s="4"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="14"/>
-      <c r="B28" s="4">
-        <f>SUM(B18:B27)</f>
-        <v>17740.72</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9819517C-B247-499C-8A9B-BF9D321254B0}">
-  <dimension ref="A1:R79"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="23.88671875" style="9" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" style="10" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="27" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="17.44140625" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="18.88671875" customWidth="1"/>
-    <col min="11" max="11" width="17.44140625" customWidth="1"/>
-    <col min="12" max="12" width="18.109375" customWidth="1"/>
-    <col min="13" max="17" width="13.6640625" customWidth="1"/>
-    <col min="18" max="18" width="22.109375" style="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="75" t="s">
+    <row r="1" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="75"/>
+      <c r="B1" s="69"/>
       <c r="D1" s="23"/>
       <c r="E1" s="24"/>
-      <c r="F1" s="68" t="s">
+      <c r="F1" s="62" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="70"/>
-    </row>
-    <row r="2" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="64"/>
+    </row>
+    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>29</v>
       </c>
@@ -3162,7 +2369,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>30</v>
       </c>
@@ -3216,7 +2423,7 @@
         <v>103343.3</v>
       </c>
     </row>
-    <row r="4" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>31</v>
       </c>
@@ -3258,7 +2465,7 @@
         <v>250227.75</v>
       </c>
     </row>
-    <row r="5" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>32</v>
       </c>
@@ -3302,7 +2509,7 @@
         <v>45350</v>
       </c>
     </row>
-    <row r="6" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>33</v>
       </c>
@@ -3346,7 +2553,7 @@
         <v>69603.87999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>34</v>
       </c>
@@ -3388,7 +2595,7 @@
         <v>25053.339999999997</v>
       </c>
     </row>
-    <row r="8" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>35</v>
       </c>
@@ -3428,7 +2635,7 @@
         <v>96808.18</v>
       </c>
     </row>
-    <row r="9" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>36</v>
       </c>
@@ -3472,7 +2679,7 @@
         <v>127257.03</v>
       </c>
     </row>
-    <row r="10" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
         <v>62</v>
       </c>
@@ -3516,7 +2723,7 @@
         <v>33334.020000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>37</v>
       </c>
@@ -3560,7 +2767,7 @@
         <v>122463.15999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>38</v>
       </c>
@@ -3602,7 +2809,7 @@
         <v>2607.3200000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>58</v>
       </c>
@@ -3646,7 +2853,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="14" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>39</v>
       </c>
@@ -3690,7 +2897,7 @@
         <v>147062</v>
       </c>
     </row>
-    <row r="15" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>40</v>
       </c>
@@ -3734,7 +2941,7 @@
         <v>122389.29999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>41</v>
       </c>
@@ -3778,7 +2985,7 @@
         <v>56615.22</v>
       </c>
     </row>
-    <row r="17" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>60</v>
       </c>
@@ -3822,7 +3029,7 @@
         <v>253279.38</v>
       </c>
     </row>
-    <row r="18" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>42</v>
       </c>
@@ -3860,7 +3067,7 @@
         <v>31041.84</v>
       </c>
     </row>
-    <row r="19" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>43</v>
       </c>
@@ -3904,7 +3111,7 @@
         <v>62981.130000000005</v>
       </c>
     </row>
-    <row r="20" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="12"/>
       <c r="B20" s="13"/>
       <c r="D20" s="41" t="s">
@@ -3944,7 +3151,7 @@
         <v>103861.32</v>
       </c>
     </row>
-    <row r="21" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>44</v>
       </c>
@@ -3986,7 +3193,7 @@
         <v>38733.25</v>
       </c>
     </row>
-    <row r="22" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>45</v>
       </c>
@@ -4020,7 +3227,7 @@
         <v>31524.93</v>
       </c>
     </row>
-    <row r="23" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>59</v>
       </c>
@@ -4064,7 +3271,7 @@
         <v>125303.81000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
         <v>46</v>
       </c>
@@ -4108,7 +3315,7 @@
         <v>193857.35</v>
       </c>
     </row>
-    <row r="25" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>47</v>
       </c>
@@ -4152,7 +3359,7 @@
         <v>79023.62</v>
       </c>
     </row>
-    <row r="26" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
         <v>48</v>
       </c>
@@ -4196,7 +3403,7 @@
         <v>84931.12999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>49</v>
       </c>
@@ -4240,7 +3447,7 @@
         <v>88333.680000000008</v>
       </c>
     </row>
-    <row r="28" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>50</v>
       </c>
@@ -4284,7 +3491,7 @@
         <v>179792.25</v>
       </c>
     </row>
-    <row r="29" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
         <v>57</v>
       </c>
@@ -4320,7 +3527,7 @@
         <v>14056.9</v>
       </c>
     </row>
-    <row r="30" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
         <v>61</v>
       </c>
@@ -4364,7 +3571,7 @@
         <v>35183.597000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>51</v>
       </c>
@@ -4402,7 +3609,7 @@
         <v>70501</v>
       </c>
     </row>
-    <row r="32" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>52</v>
       </c>
@@ -4444,7 +3651,7 @@
         <v>219829.37</v>
       </c>
     </row>
-    <row r="33" spans="1:18" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>53</v>
       </c>
@@ -4488,7 +3695,7 @@
         <v>12186.71</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>54</v>
       </c>
@@ -4524,7 +3731,7 @@
         <v>17502</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>67</v>
       </c>
@@ -4562,7 +3769,7 @@
         <v>43485.59</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>66</v>
       </c>
@@ -4594,7 +3801,7 @@
         <v>3400.78</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
         <v>55</v>
       </c>
@@ -4639,7 +3846,7 @@
         <v>121149.51000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
         <v>63</v>
       </c>
@@ -4681,7 +3888,7 @@
         <v>166368.10999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="21"/>
       <c r="B39" s="22"/>
       <c r="D39" s="41" t="s">
@@ -4721,7 +3928,7 @@
         <v>78975.91</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="21"/>
       <c r="B40" s="22"/>
       <c r="D40" s="45" t="s">
@@ -4753,7 +3960,7 @@
         <v>152258.96000000002</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="21"/>
       <c r="B41" s="22"/>
       <c r="D41" s="45" t="s">
@@ -4785,7 +3992,7 @@
         <v>20000.010000000002</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="21"/>
       <c r="B42" s="22"/>
       <c r="D42" s="45" t="s">
@@ -4821,7 +4028,7 @@
         <v>30306.400000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="21"/>
       <c r="B43" s="22"/>
       <c r="D43" s="45" t="s">
@@ -4859,7 +4066,7 @@
         <v>65961</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="21"/>
       <c r="B44" s="22"/>
       <c r="D44" s="45" t="s">
@@ -4897,11 +4104,11 @@
         <v>101856.02</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="21"/>
       <c r="B45" s="22"/>
       <c r="D45" s="45" t="s">
-        <v>162</v>
+        <v>135</v>
       </c>
       <c r="E45" s="42">
         <v>156000</v>
@@ -4933,11 +4140,11 @@
         <v>148691.04999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="21"/>
       <c r="B46" s="22"/>
       <c r="D46" s="45" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
       <c r="E46" s="42">
         <v>90000</v>
@@ -4969,11 +4176,11 @@
         <v>66280.149999999994</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="21"/>
       <c r="B47" s="22"/>
       <c r="D47" s="45" t="s">
-        <v>166</v>
+        <v>137</v>
       </c>
       <c r="E47" s="42">
         <v>0</v>
@@ -5001,11 +4208,11 @@
         <v>19573.560000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="21"/>
       <c r="B48" s="22"/>
       <c r="D48" s="45" t="s">
-        <v>178</v>
+        <v>138</v>
       </c>
       <c r="E48" s="42">
         <v>18000</v>
@@ -5037,11 +4244,11 @@
         <v>19925.34</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="21"/>
       <c r="B49" s="22"/>
       <c r="D49" s="45" t="s">
-        <v>193</v>
+        <v>139</v>
       </c>
       <c r="E49" s="42">
         <v>50000</v>
@@ -5069,7 +4276,7 @@
         <v>18025.53</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="21"/>
       <c r="B50" s="22"/>
       <c r="D50" s="45"/>
@@ -5095,7 +4302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="21"/>
       <c r="B51" s="22"/>
       <c r="D51" s="45"/>
@@ -5121,13 +4328,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="21"/>
       <c r="B52" s="22"/>
-      <c r="D52" s="76" t="s">
+      <c r="D52" s="70" t="s">
         <v>119</v>
       </c>
-      <c r="E52" s="77"/>
+      <c r="E52" s="71"/>
       <c r="F52" s="48">
         <f t="shared" ref="F52:Q52" si="4">SUM(F3:F51)</f>
         <v>376464.647</v>
@@ -5181,66 +4388,66 @@
         <v>3970297.6869999995</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="21"/>
       <c r="B53" s="22"/>
-      <c r="D53" s="80"/>
-      <c r="E53" s="81"/>
-      <c r="F53" s="82"/>
-      <c r="G53" s="83"/>
-      <c r="H53" s="83"/>
-      <c r="I53" s="83"/>
-      <c r="J53" s="83"/>
-      <c r="K53" s="83"/>
-      <c r="L53" s="83"/>
-      <c r="M53" s="83"/>
-      <c r="N53" s="83"/>
-      <c r="O53" s="83"/>
-      <c r="P53" s="83"/>
-      <c r="Q53" s="83"/>
-      <c r="R53" s="84"/>
-    </row>
-    <row r="54" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D53" s="74"/>
+      <c r="E53" s="75"/>
+      <c r="F53" s="76"/>
+      <c r="G53" s="77"/>
+      <c r="H53" s="77"/>
+      <c r="I53" s="77"/>
+      <c r="J53" s="77"/>
+      <c r="K53" s="77"/>
+      <c r="L53" s="77"/>
+      <c r="M53" s="77"/>
+      <c r="N53" s="77"/>
+      <c r="O53" s="77"/>
+      <c r="P53" s="77"/>
+      <c r="Q53" s="77"/>
+      <c r="R53" s="78"/>
+    </row>
+    <row r="54" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="21"/>
       <c r="B54" s="22"/>
-      <c r="D54" s="78" t="s">
+      <c r="D54" s="72" t="s">
         <v>124</v>
       </c>
-      <c r="E54" s="79"/>
-      <c r="F54" s="85"/>
-      <c r="G54" s="85"/>
-      <c r="H54" s="85"/>
-      <c r="I54" s="85"/>
-      <c r="J54" s="85"/>
-      <c r="K54" s="85"/>
-      <c r="L54" s="85"/>
-      <c r="M54" s="85"/>
-      <c r="N54" s="85"/>
-      <c r="O54" s="85"/>
-      <c r="P54" s="85"/>
-      <c r="Q54" s="85"/>
-      <c r="R54" s="86"/>
-    </row>
-    <row r="55" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="73"/>
-      <c r="B55" s="74"/>
-      <c r="D55" s="71"/>
-      <c r="E55" s="72"/>
-      <c r="F55" s="85"/>
-      <c r="G55" s="85"/>
-      <c r="H55" s="85"/>
-      <c r="I55" s="85"/>
-      <c r="J55" s="85"/>
-      <c r="K55" s="85"/>
-      <c r="L55" s="85"/>
-      <c r="M55" s="85"/>
-      <c r="N55" s="85"/>
-      <c r="O55" s="85"/>
-      <c r="P55" s="85"/>
-      <c r="Q55" s="85"/>
-      <c r="R55" s="86"/>
-    </row>
-    <row r="56" spans="1:18" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E54" s="73"/>
+      <c r="F54" s="79"/>
+      <c r="G54" s="79"/>
+      <c r="H54" s="79"/>
+      <c r="I54" s="79"/>
+      <c r="J54" s="79"/>
+      <c r="K54" s="79"/>
+      <c r="L54" s="79"/>
+      <c r="M54" s="79"/>
+      <c r="N54" s="79"/>
+      <c r="O54" s="79"/>
+      <c r="P54" s="79"/>
+      <c r="Q54" s="79"/>
+      <c r="R54" s="80"/>
+    </row>
+    <row r="55" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="67"/>
+      <c r="B55" s="68"/>
+      <c r="D55" s="65"/>
+      <c r="E55" s="66"/>
+      <c r="F55" s="79"/>
+      <c r="G55" s="79"/>
+      <c r="H55" s="79"/>
+      <c r="I55" s="79"/>
+      <c r="J55" s="79"/>
+      <c r="K55" s="79"/>
+      <c r="L55" s="79"/>
+      <c r="M55" s="79"/>
+      <c r="N55" s="79"/>
+      <c r="O55" s="79"/>
+      <c r="P55" s="79"/>
+      <c r="Q55" s="79"/>
+      <c r="R55" s="80"/>
+    </row>
+    <row r="56" spans="1:18" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="19" t="s">
         <v>64</v>
       </c>
@@ -5254,38 +4461,38 @@
       <c r="E56" s="35">
         <v>3100997.78</v>
       </c>
-      <c r="F56" s="85"/>
-      <c r="G56" s="85"/>
-      <c r="H56" s="85"/>
-      <c r="I56" s="85"/>
-      <c r="J56" s="85"/>
-      <c r="K56" s="85"/>
-      <c r="L56" s="85"/>
-      <c r="M56" s="85"/>
-      <c r="N56" s="85"/>
-      <c r="O56" s="85"/>
-      <c r="P56" s="85"/>
-      <c r="Q56" s="85"/>
-      <c r="R56" s="86"/>
-    </row>
-    <row r="57" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D57" s="87"/>
-      <c r="E57" s="88"/>
-      <c r="F57" s="85"/>
-      <c r="G57" s="85"/>
-      <c r="H57" s="85"/>
-      <c r="I57" s="85"/>
-      <c r="J57" s="85"/>
-      <c r="K57" s="85"/>
-      <c r="L57" s="85"/>
-      <c r="M57" s="85"/>
-      <c r="N57" s="85"/>
-      <c r="O57" s="85"/>
-      <c r="P57" s="85"/>
-      <c r="Q57" s="85"/>
-      <c r="R57" s="86"/>
-    </row>
-    <row r="58" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F56" s="79"/>
+      <c r="G56" s="79"/>
+      <c r="H56" s="79"/>
+      <c r="I56" s="79"/>
+      <c r="J56" s="79"/>
+      <c r="K56" s="79"/>
+      <c r="L56" s="79"/>
+      <c r="M56" s="79"/>
+      <c r="N56" s="79"/>
+      <c r="O56" s="79"/>
+      <c r="P56" s="79"/>
+      <c r="Q56" s="79"/>
+      <c r="R56" s="80"/>
+    </row>
+    <row r="57" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D57" s="81"/>
+      <c r="E57" s="82"/>
+      <c r="F57" s="79"/>
+      <c r="G57" s="79"/>
+      <c r="H57" s="79"/>
+      <c r="I57" s="79"/>
+      <c r="J57" s="79"/>
+      <c r="K57" s="79"/>
+      <c r="L57" s="79"/>
+      <c r="M57" s="79"/>
+      <c r="N57" s="79"/>
+      <c r="O57" s="79"/>
+      <c r="P57" s="79"/>
+      <c r="Q57" s="79"/>
+      <c r="R57" s="80"/>
+    </row>
+    <row r="58" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D58" s="36" t="s">
         <v>129</v>
       </c>
@@ -5293,38 +4500,38 @@
         <f>SUM(E3:E51)</f>
         <v>6816000</v>
       </c>
-      <c r="F58" s="85"/>
-      <c r="G58" s="85"/>
-      <c r="H58" s="85"/>
-      <c r="I58" s="85"/>
-      <c r="J58" s="85"/>
-      <c r="K58" s="85"/>
-      <c r="L58" s="85"/>
-      <c r="M58" s="85"/>
-      <c r="N58" s="85"/>
-      <c r="O58" s="85"/>
-      <c r="P58" s="85"/>
-      <c r="Q58" s="85"/>
-      <c r="R58" s="86"/>
-    </row>
-    <row r="59" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F58" s="79"/>
+      <c r="G58" s="79"/>
+      <c r="H58" s="79"/>
+      <c r="I58" s="79"/>
+      <c r="J58" s="79"/>
+      <c r="K58" s="79"/>
+      <c r="L58" s="79"/>
+      <c r="M58" s="79"/>
+      <c r="N58" s="79"/>
+      <c r="O58" s="79"/>
+      <c r="P58" s="79"/>
+      <c r="Q58" s="79"/>
+      <c r="R58" s="80"/>
+    </row>
+    <row r="59" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D59" s="32"/>
       <c r="E59" s="33"/>
-      <c r="F59" s="85"/>
-      <c r="G59" s="85"/>
-      <c r="H59" s="85"/>
-      <c r="I59" s="85"/>
-      <c r="J59" s="85"/>
-      <c r="K59" s="85"/>
-      <c r="L59" s="85"/>
-      <c r="M59" s="85"/>
-      <c r="N59" s="85"/>
-      <c r="O59" s="85"/>
-      <c r="P59" s="85"/>
-      <c r="Q59" s="85"/>
-      <c r="R59" s="86"/>
-    </row>
-    <row r="60" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F59" s="79"/>
+      <c r="G59" s="79"/>
+      <c r="H59" s="79"/>
+      <c r="I59" s="79"/>
+      <c r="J59" s="79"/>
+      <c r="K59" s="79"/>
+      <c r="L59" s="79"/>
+      <c r="M59" s="79"/>
+      <c r="N59" s="79"/>
+      <c r="O59" s="79"/>
+      <c r="P59" s="79"/>
+      <c r="Q59" s="79"/>
+      <c r="R59" s="80"/>
+    </row>
+    <row r="60" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D60" s="30" t="s">
         <v>130</v>
       </c>
@@ -5332,345 +4539,345 @@
         <f>SUM(E58-E56)</f>
         <v>3715002.22</v>
       </c>
-      <c r="F60" s="85"/>
-      <c r="G60" s="85"/>
-      <c r="H60" s="85"/>
-      <c r="I60" s="85"/>
-      <c r="J60" s="85"/>
-      <c r="K60" s="85"/>
-      <c r="L60" s="85"/>
-      <c r="M60" s="85"/>
-      <c r="N60" s="85"/>
-      <c r="O60" s="85"/>
-      <c r="P60" s="85"/>
-      <c r="Q60" s="85"/>
-      <c r="R60" s="86"/>
-    </row>
-    <row r="61" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D61" s="89"/>
-      <c r="E61" s="90"/>
-      <c r="F61" s="85"/>
-      <c r="G61" s="85"/>
-      <c r="H61" s="85"/>
-      <c r="I61" s="85"/>
-      <c r="J61" s="85"/>
-      <c r="K61" s="85"/>
-      <c r="L61" s="85"/>
-      <c r="M61" s="85"/>
-      <c r="N61" s="85"/>
-      <c r="O61" s="85"/>
-      <c r="P61" s="85"/>
-      <c r="Q61" s="85"/>
-      <c r="R61" s="86"/>
-    </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="D62" s="64"/>
-      <c r="E62" s="64"/>
-      <c r="F62" s="64"/>
-      <c r="G62" s="64"/>
-      <c r="H62" s="64"/>
-      <c r="I62" s="64"/>
-      <c r="J62" s="64"/>
-      <c r="K62" s="64"/>
-      <c r="L62" s="64"/>
-      <c r="M62" s="64"/>
-      <c r="N62" s="64"/>
-      <c r="O62" s="64"/>
-      <c r="P62" s="64"/>
-      <c r="Q62" s="64"/>
-      <c r="R62" s="65"/>
-    </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="D63" s="66"/>
-      <c r="E63" s="66"/>
-      <c r="F63" s="66"/>
-      <c r="G63" s="66"/>
-      <c r="H63" s="66"/>
-      <c r="I63" s="66"/>
-      <c r="J63" s="66"/>
-      <c r="K63" s="66"/>
-      <c r="L63" s="66"/>
-      <c r="M63" s="66"/>
-      <c r="N63" s="66"/>
-      <c r="O63" s="66"/>
-      <c r="P63" s="66"/>
-      <c r="Q63" s="66"/>
-      <c r="R63" s="67"/>
-    </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="D64" s="66"/>
-      <c r="E64" s="66"/>
-      <c r="F64" s="66"/>
-      <c r="G64" s="66"/>
-      <c r="H64" s="66"/>
-      <c r="I64" s="66"/>
-      <c r="J64" s="66"/>
-      <c r="K64" s="66"/>
-      <c r="L64" s="66"/>
-      <c r="M64" s="66"/>
-      <c r="N64" s="66"/>
-      <c r="O64" s="66"/>
-      <c r="P64" s="66"/>
-      <c r="Q64" s="66"/>
-      <c r="R64" s="67"/>
-    </row>
-    <row r="65" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D65" s="66"/>
-      <c r="E65" s="66"/>
-      <c r="F65" s="66"/>
-      <c r="G65" s="66"/>
-      <c r="H65" s="66"/>
-      <c r="I65" s="66"/>
-      <c r="J65" s="66"/>
-      <c r="K65" s="66"/>
-      <c r="L65" s="66"/>
-      <c r="M65" s="66"/>
-      <c r="N65" s="66"/>
-      <c r="O65" s="66"/>
-      <c r="P65" s="66"/>
-      <c r="Q65" s="66"/>
-      <c r="R65" s="67"/>
-    </row>
-    <row r="66" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D66" s="66"/>
-      <c r="E66" s="66"/>
-      <c r="F66" s="66"/>
-      <c r="G66" s="66"/>
-      <c r="H66" s="66"/>
-      <c r="I66" s="66"/>
-      <c r="J66" s="66"/>
-      <c r="K66" s="66"/>
-      <c r="L66" s="66"/>
-      <c r="M66" s="66"/>
-      <c r="N66" s="66"/>
-      <c r="O66" s="66"/>
-      <c r="P66" s="66"/>
-      <c r="Q66" s="66"/>
-      <c r="R66" s="67"/>
-    </row>
-    <row r="67" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D67" s="66"/>
-      <c r="E67" s="66"/>
-      <c r="F67" s="66"/>
-      <c r="G67" s="66"/>
-      <c r="H67" s="66"/>
-      <c r="I67" s="66"/>
-      <c r="J67" s="66"/>
-      <c r="K67" s="66"/>
-      <c r="L67" s="66"/>
-      <c r="M67" s="66"/>
-      <c r="N67" s="66"/>
-      <c r="O67" s="66"/>
-      <c r="P67" s="66"/>
-      <c r="Q67" s="66"/>
-      <c r="R67" s="67"/>
-    </row>
-    <row r="68" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D68" s="66"/>
-      <c r="E68" s="66"/>
-      <c r="F68" s="66"/>
-      <c r="G68" s="66"/>
-      <c r="H68" s="66"/>
-      <c r="I68" s="66"/>
-      <c r="J68" s="66"/>
-      <c r="K68" s="66"/>
-      <c r="L68" s="66"/>
-      <c r="M68" s="66"/>
-      <c r="N68" s="66"/>
-      <c r="O68" s="66"/>
-      <c r="P68" s="66"/>
-      <c r="Q68" s="66"/>
-      <c r="R68" s="67"/>
-    </row>
-    <row r="69" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D69" s="66"/>
-      <c r="E69" s="66"/>
-      <c r="F69" s="66"/>
-      <c r="G69" s="66"/>
-      <c r="H69" s="66"/>
-      <c r="I69" s="66"/>
-      <c r="J69" s="66"/>
-      <c r="K69" s="66"/>
-      <c r="L69" s="66"/>
-      <c r="M69" s="66"/>
-      <c r="N69" s="66"/>
-      <c r="O69" s="66"/>
-      <c r="P69" s="66"/>
-      <c r="Q69" s="66"/>
-      <c r="R69" s="67"/>
-    </row>
-    <row r="70" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D70" s="66"/>
-      <c r="E70" s="66"/>
-      <c r="F70" s="66"/>
-      <c r="G70" s="66"/>
-      <c r="H70" s="66"/>
-      <c r="I70" s="66"/>
-      <c r="J70" s="66"/>
-      <c r="K70" s="66"/>
-      <c r="L70" s="66"/>
-      <c r="M70" s="66"/>
-      <c r="N70" s="66"/>
-      <c r="O70" s="66"/>
-      <c r="P70" s="66"/>
-      <c r="Q70" s="66"/>
-      <c r="R70" s="67"/>
-    </row>
-    <row r="71" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D71" s="66"/>
-      <c r="E71" s="66"/>
-      <c r="F71" s="66"/>
-      <c r="G71" s="66"/>
-      <c r="H71" s="66"/>
-      <c r="I71" s="66"/>
-      <c r="J71" s="66"/>
-      <c r="K71" s="66"/>
-      <c r="L71" s="66"/>
-      <c r="M71" s="66"/>
-      <c r="N71" s="66"/>
-      <c r="O71" s="66"/>
-      <c r="P71" s="66"/>
-      <c r="Q71" s="66"/>
-      <c r="R71" s="67"/>
-    </row>
-    <row r="72" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D72" s="66"/>
-      <c r="E72" s="66"/>
-      <c r="F72" s="66"/>
-      <c r="G72" s="66"/>
-      <c r="H72" s="66"/>
-      <c r="I72" s="66"/>
-      <c r="J72" s="66"/>
-      <c r="K72" s="66"/>
-      <c r="L72" s="66"/>
-      <c r="M72" s="66"/>
-      <c r="N72" s="66"/>
-      <c r="O72" s="66"/>
-      <c r="P72" s="66"/>
-      <c r="Q72" s="66"/>
-      <c r="R72" s="67"/>
-    </row>
-    <row r="73" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D73" s="66"/>
-      <c r="E73" s="66"/>
-      <c r="F73" s="66"/>
-      <c r="G73" s="66"/>
-      <c r="H73" s="66"/>
-      <c r="I73" s="66"/>
-      <c r="J73" s="66"/>
-      <c r="K73" s="66"/>
-      <c r="L73" s="66"/>
-      <c r="M73" s="66"/>
-      <c r="N73" s="66"/>
-      <c r="O73" s="66"/>
-      <c r="P73" s="66"/>
-      <c r="Q73" s="66"/>
-      <c r="R73" s="67"/>
-    </row>
-    <row r="74" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D74" s="66"/>
-      <c r="E74" s="66"/>
-      <c r="F74" s="66"/>
-      <c r="G74" s="66"/>
-      <c r="H74" s="66"/>
-      <c r="I74" s="66"/>
-      <c r="J74" s="66"/>
-      <c r="K74" s="66"/>
-      <c r="L74" s="66"/>
-      <c r="M74" s="66"/>
-      <c r="N74" s="66"/>
-      <c r="O74" s="66"/>
-      <c r="P74" s="66"/>
-      <c r="Q74" s="66"/>
-      <c r="R74" s="67"/>
-    </row>
-    <row r="75" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D75" s="66"/>
-      <c r="E75" s="66"/>
-      <c r="F75" s="66"/>
-      <c r="G75" s="66"/>
-      <c r="H75" s="66"/>
-      <c r="I75" s="66"/>
-      <c r="J75" s="66"/>
-      <c r="K75" s="66"/>
-      <c r="L75" s="66"/>
-      <c r="M75" s="66"/>
-      <c r="N75" s="66"/>
-      <c r="O75" s="66"/>
-      <c r="P75" s="66"/>
-      <c r="Q75" s="66"/>
-      <c r="R75" s="67"/>
-    </row>
-    <row r="76" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D76" s="66"/>
-      <c r="E76" s="66"/>
-      <c r="F76" s="66"/>
-      <c r="G76" s="66"/>
-      <c r="H76" s="66"/>
-      <c r="I76" s="66"/>
-      <c r="J76" s="66"/>
-      <c r="K76" s="66"/>
-      <c r="L76" s="66"/>
-      <c r="M76" s="66"/>
-      <c r="N76" s="66"/>
-      <c r="O76" s="66"/>
-      <c r="P76" s="66"/>
-      <c r="Q76" s="66"/>
-      <c r="R76" s="67"/>
-    </row>
-    <row r="77" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D77" s="66"/>
-      <c r="E77" s="66"/>
-      <c r="F77" s="66"/>
-      <c r="G77" s="66"/>
-      <c r="H77" s="66"/>
-      <c r="I77" s="66"/>
-      <c r="J77" s="66"/>
-      <c r="K77" s="66"/>
-      <c r="L77" s="66"/>
-      <c r="M77" s="66"/>
-      <c r="N77" s="66"/>
-      <c r="O77" s="66"/>
-      <c r="P77" s="66"/>
-      <c r="Q77" s="66"/>
-      <c r="R77" s="67"/>
-    </row>
-    <row r="78" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D78" s="66"/>
-      <c r="E78" s="66"/>
-      <c r="F78" s="66"/>
-      <c r="G78" s="66"/>
-      <c r="H78" s="66"/>
-      <c r="I78" s="66"/>
-      <c r="J78" s="66"/>
-      <c r="K78" s="66"/>
-      <c r="L78" s="66"/>
-      <c r="M78" s="66"/>
-      <c r="N78" s="66"/>
-      <c r="O78" s="66"/>
-      <c r="P78" s="66"/>
-      <c r="Q78" s="66"/>
-      <c r="R78" s="67"/>
-    </row>
-    <row r="79" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D79" s="66"/>
-      <c r="E79" s="66"/>
-      <c r="F79" s="66"/>
-      <c r="G79" s="66"/>
-      <c r="H79" s="66"/>
-      <c r="I79" s="66"/>
-      <c r="J79" s="66"/>
-      <c r="K79" s="66"/>
-      <c r="L79" s="66"/>
-      <c r="M79" s="66"/>
-      <c r="N79" s="66"/>
-      <c r="O79" s="66"/>
-      <c r="P79" s="66"/>
-      <c r="Q79" s="66"/>
-      <c r="R79" s="67"/>
+      <c r="F60" s="79"/>
+      <c r="G60" s="79"/>
+      <c r="H60" s="79"/>
+      <c r="I60" s="79"/>
+      <c r="J60" s="79"/>
+      <c r="K60" s="79"/>
+      <c r="L60" s="79"/>
+      <c r="M60" s="79"/>
+      <c r="N60" s="79"/>
+      <c r="O60" s="79"/>
+      <c r="P60" s="79"/>
+      <c r="Q60" s="79"/>
+      <c r="R60" s="80"/>
+    </row>
+    <row r="61" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D61" s="83"/>
+      <c r="E61" s="84"/>
+      <c r="F61" s="79"/>
+      <c r="G61" s="79"/>
+      <c r="H61" s="79"/>
+      <c r="I61" s="79"/>
+      <c r="J61" s="79"/>
+      <c r="K61" s="79"/>
+      <c r="L61" s="79"/>
+      <c r="M61" s="79"/>
+      <c r="N61" s="79"/>
+      <c r="O61" s="79"/>
+      <c r="P61" s="79"/>
+      <c r="Q61" s="79"/>
+      <c r="R61" s="80"/>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D62" s="58"/>
+      <c r="E62" s="58"/>
+      <c r="F62" s="58"/>
+      <c r="G62" s="58"/>
+      <c r="H62" s="58"/>
+      <c r="I62" s="58"/>
+      <c r="J62" s="58"/>
+      <c r="K62" s="58"/>
+      <c r="L62" s="58"/>
+      <c r="M62" s="58"/>
+      <c r="N62" s="58"/>
+      <c r="O62" s="58"/>
+      <c r="P62" s="58"/>
+      <c r="Q62" s="58"/>
+      <c r="R62" s="59"/>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D63" s="60"/>
+      <c r="E63" s="60"/>
+      <c r="F63" s="60"/>
+      <c r="G63" s="60"/>
+      <c r="H63" s="60"/>
+      <c r="I63" s="60"/>
+      <c r="J63" s="60"/>
+      <c r="K63" s="60"/>
+      <c r="L63" s="60"/>
+      <c r="M63" s="60"/>
+      <c r="N63" s="60"/>
+      <c r="O63" s="60"/>
+      <c r="P63" s="60"/>
+      <c r="Q63" s="60"/>
+      <c r="R63" s="61"/>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D64" s="60"/>
+      <c r="E64" s="60"/>
+      <c r="F64" s="60"/>
+      <c r="G64" s="60"/>
+      <c r="H64" s="60"/>
+      <c r="I64" s="60"/>
+      <c r="J64" s="60"/>
+      <c r="K64" s="60"/>
+      <c r="L64" s="60"/>
+      <c r="M64" s="60"/>
+      <c r="N64" s="60"/>
+      <c r="O64" s="60"/>
+      <c r="P64" s="60"/>
+      <c r="Q64" s="60"/>
+      <c r="R64" s="61"/>
+    </row>
+    <row r="65" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D65" s="60"/>
+      <c r="E65" s="60"/>
+      <c r="F65" s="60"/>
+      <c r="G65" s="60"/>
+      <c r="H65" s="60"/>
+      <c r="I65" s="60"/>
+      <c r="J65" s="60"/>
+      <c r="K65" s="60"/>
+      <c r="L65" s="60"/>
+      <c r="M65" s="60"/>
+      <c r="N65" s="60"/>
+      <c r="O65" s="60"/>
+      <c r="P65" s="60"/>
+      <c r="Q65" s="60"/>
+      <c r="R65" s="61"/>
+    </row>
+    <row r="66" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D66" s="60"/>
+      <c r="E66" s="60"/>
+      <c r="F66" s="60"/>
+      <c r="G66" s="60"/>
+      <c r="H66" s="60"/>
+      <c r="I66" s="60"/>
+      <c r="J66" s="60"/>
+      <c r="K66" s="60"/>
+      <c r="L66" s="60"/>
+      <c r="M66" s="60"/>
+      <c r="N66" s="60"/>
+      <c r="O66" s="60"/>
+      <c r="P66" s="60"/>
+      <c r="Q66" s="60"/>
+      <c r="R66" s="61"/>
+    </row>
+    <row r="67" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D67" s="60"/>
+      <c r="E67" s="60"/>
+      <c r="F67" s="60"/>
+      <c r="G67" s="60"/>
+      <c r="H67" s="60"/>
+      <c r="I67" s="60"/>
+      <c r="J67" s="60"/>
+      <c r="K67" s="60"/>
+      <c r="L67" s="60"/>
+      <c r="M67" s="60"/>
+      <c r="N67" s="60"/>
+      <c r="O67" s="60"/>
+      <c r="P67" s="60"/>
+      <c r="Q67" s="60"/>
+      <c r="R67" s="61"/>
+    </row>
+    <row r="68" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D68" s="60"/>
+      <c r="E68" s="60"/>
+      <c r="F68" s="60"/>
+      <c r="G68" s="60"/>
+      <c r="H68" s="60"/>
+      <c r="I68" s="60"/>
+      <c r="J68" s="60"/>
+      <c r="K68" s="60"/>
+      <c r="L68" s="60"/>
+      <c r="M68" s="60"/>
+      <c r="N68" s="60"/>
+      <c r="O68" s="60"/>
+      <c r="P68" s="60"/>
+      <c r="Q68" s="60"/>
+      <c r="R68" s="61"/>
+    </row>
+    <row r="69" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D69" s="60"/>
+      <c r="E69" s="60"/>
+      <c r="F69" s="60"/>
+      <c r="G69" s="60"/>
+      <c r="H69" s="60"/>
+      <c r="I69" s="60"/>
+      <c r="J69" s="60"/>
+      <c r="K69" s="60"/>
+      <c r="L69" s="60"/>
+      <c r="M69" s="60"/>
+      <c r="N69" s="60"/>
+      <c r="O69" s="60"/>
+      <c r="P69" s="60"/>
+      <c r="Q69" s="60"/>
+      <c r="R69" s="61"/>
+    </row>
+    <row r="70" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D70" s="60"/>
+      <c r="E70" s="60"/>
+      <c r="F70" s="60"/>
+      <c r="G70" s="60"/>
+      <c r="H70" s="60"/>
+      <c r="I70" s="60"/>
+      <c r="J70" s="60"/>
+      <c r="K70" s="60"/>
+      <c r="L70" s="60"/>
+      <c r="M70" s="60"/>
+      <c r="N70" s="60"/>
+      <c r="O70" s="60"/>
+      <c r="P70" s="60"/>
+      <c r="Q70" s="60"/>
+      <c r="R70" s="61"/>
+    </row>
+    <row r="71" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D71" s="60"/>
+      <c r="E71" s="60"/>
+      <c r="F71" s="60"/>
+      <c r="G71" s="60"/>
+      <c r="H71" s="60"/>
+      <c r="I71" s="60"/>
+      <c r="J71" s="60"/>
+      <c r="K71" s="60"/>
+      <c r="L71" s="60"/>
+      <c r="M71" s="60"/>
+      <c r="N71" s="60"/>
+      <c r="O71" s="60"/>
+      <c r="P71" s="60"/>
+      <c r="Q71" s="60"/>
+      <c r="R71" s="61"/>
+    </row>
+    <row r="72" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D72" s="60"/>
+      <c r="E72" s="60"/>
+      <c r="F72" s="60"/>
+      <c r="G72" s="60"/>
+      <c r="H72" s="60"/>
+      <c r="I72" s="60"/>
+      <c r="J72" s="60"/>
+      <c r="K72" s="60"/>
+      <c r="L72" s="60"/>
+      <c r="M72" s="60"/>
+      <c r="N72" s="60"/>
+      <c r="O72" s="60"/>
+      <c r="P72" s="60"/>
+      <c r="Q72" s="60"/>
+      <c r="R72" s="61"/>
+    </row>
+    <row r="73" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D73" s="60"/>
+      <c r="E73" s="60"/>
+      <c r="F73" s="60"/>
+      <c r="G73" s="60"/>
+      <c r="H73" s="60"/>
+      <c r="I73" s="60"/>
+      <c r="J73" s="60"/>
+      <c r="K73" s="60"/>
+      <c r="L73" s="60"/>
+      <c r="M73" s="60"/>
+      <c r="N73" s="60"/>
+      <c r="O73" s="60"/>
+      <c r="P73" s="60"/>
+      <c r="Q73" s="60"/>
+      <c r="R73" s="61"/>
+    </row>
+    <row r="74" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D74" s="60"/>
+      <c r="E74" s="60"/>
+      <c r="F74" s="60"/>
+      <c r="G74" s="60"/>
+      <c r="H74" s="60"/>
+      <c r="I74" s="60"/>
+      <c r="J74" s="60"/>
+      <c r="K74" s="60"/>
+      <c r="L74" s="60"/>
+      <c r="M74" s="60"/>
+      <c r="N74" s="60"/>
+      <c r="O74" s="60"/>
+      <c r="P74" s="60"/>
+      <c r="Q74" s="60"/>
+      <c r="R74" s="61"/>
+    </row>
+    <row r="75" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D75" s="60"/>
+      <c r="E75" s="60"/>
+      <c r="F75" s="60"/>
+      <c r="G75" s="60"/>
+      <c r="H75" s="60"/>
+      <c r="I75" s="60"/>
+      <c r="J75" s="60"/>
+      <c r="K75" s="60"/>
+      <c r="L75" s="60"/>
+      <c r="M75" s="60"/>
+      <c r="N75" s="60"/>
+      <c r="O75" s="60"/>
+      <c r="P75" s="60"/>
+      <c r="Q75" s="60"/>
+      <c r="R75" s="61"/>
+    </row>
+    <row r="76" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D76" s="60"/>
+      <c r="E76" s="60"/>
+      <c r="F76" s="60"/>
+      <c r="G76" s="60"/>
+      <c r="H76" s="60"/>
+      <c r="I76" s="60"/>
+      <c r="J76" s="60"/>
+      <c r="K76" s="60"/>
+      <c r="L76" s="60"/>
+      <c r="M76" s="60"/>
+      <c r="N76" s="60"/>
+      <c r="O76" s="60"/>
+      <c r="P76" s="60"/>
+      <c r="Q76" s="60"/>
+      <c r="R76" s="61"/>
+    </row>
+    <row r="77" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D77" s="60"/>
+      <c r="E77" s="60"/>
+      <c r="F77" s="60"/>
+      <c r="G77" s="60"/>
+      <c r="H77" s="60"/>
+      <c r="I77" s="60"/>
+      <c r="J77" s="60"/>
+      <c r="K77" s="60"/>
+      <c r="L77" s="60"/>
+      <c r="M77" s="60"/>
+      <c r="N77" s="60"/>
+      <c r="O77" s="60"/>
+      <c r="P77" s="60"/>
+      <c r="Q77" s="60"/>
+      <c r="R77" s="61"/>
+    </row>
+    <row r="78" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D78" s="60"/>
+      <c r="E78" s="60"/>
+      <c r="F78" s="60"/>
+      <c r="G78" s="60"/>
+      <c r="H78" s="60"/>
+      <c r="I78" s="60"/>
+      <c r="J78" s="60"/>
+      <c r="K78" s="60"/>
+      <c r="L78" s="60"/>
+      <c r="M78" s="60"/>
+      <c r="N78" s="60"/>
+      <c r="O78" s="60"/>
+      <c r="P78" s="60"/>
+      <c r="Q78" s="60"/>
+      <c r="R78" s="61"/>
+    </row>
+    <row r="79" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D79" s="60"/>
+      <c r="E79" s="60"/>
+      <c r="F79" s="60"/>
+      <c r="G79" s="60"/>
+      <c r="H79" s="60"/>
+      <c r="I79" s="60"/>
+      <c r="J79" s="60"/>
+      <c r="K79" s="60"/>
+      <c r="L79" s="60"/>
+      <c r="M79" s="60"/>
+      <c r="N79" s="60"/>
+      <c r="O79" s="60"/>
+      <c r="P79" s="60"/>
+      <c r="Q79" s="60"/>
+      <c r="R79" s="61"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D1:R44">
+  <sortState ref="D1:R44">
     <sortCondition ref="D3:D40"/>
   </sortState>
   <mergeCells count="11">
@@ -5692,389 +4899,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CC7D116-6FB4-42D9-AF3D-72DD83D3A496}">
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.109375" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="4">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B3" s="4">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="B4" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="B7" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="B8" s="4">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
-      <c r="B9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
-      <c r="B10" s="4">
-        <f>SUM(B1:B9)</f>
-        <v>46000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="B14" s="4">
-        <v>450</v>
-      </c>
-      <c r="C14" s="14">
-        <v>40</v>
-      </c>
-      <c r="D14" s="4">
-        <f>B14*C14</f>
-        <v>18000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="B15" s="4">
-        <v>100</v>
-      </c>
-      <c r="C15" s="14">
-        <v>40</v>
-      </c>
-      <c r="D15" s="4">
-        <f t="shared" ref="D15:D17" si="0">B15*C15</f>
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="B16" s="4">
-        <v>285</v>
-      </c>
-      <c r="C16" s="14">
-        <v>40</v>
-      </c>
-      <c r="D16" s="4">
-        <f t="shared" si="0"/>
-        <v>11400</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="B17" s="4">
-        <v>160</v>
-      </c>
-      <c r="C17" s="14">
-        <v>40</v>
-      </c>
-      <c r="D17" s="4">
-        <f t="shared" si="0"/>
-        <v>6400</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="4">
-        <v>5335</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="4">
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="4">
-        <f>SUM(D14:D19)</f>
-        <v>57135</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87B95A1E-1B97-447C-AF61-5B18B0EA5D22}">
-  <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="B1" s="4">
-        <v>24000</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="4">
-        <v>96000</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="14"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="14"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="14"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="14"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="14"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="14"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="14"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="14"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="14"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="14"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="14"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="14"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="14"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="14"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="14"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="14"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="14"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="14"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="14"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="14"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="14"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="14"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="14"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="14"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="14"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="14"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="14"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="14"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="14"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="14"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="14"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="14"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="14"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="14"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="14"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="14"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="14"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="14"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6804ECC8-52CB-4248-93E7-8E968796D793}">
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="59.33203125" customWidth="1"/>
+    <col min="1" max="1" width="59.28515625" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>133</v>
       </c>
@@ -6088,7 +4922,7 @@
       <c r="G1" s="14"/>
       <c r="H1" s="14"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14"/>
       <c r="B2" s="14"/>
       <c r="C2" s="49">
@@ -6100,7 +4934,7 @@
       <c r="G2" s="14"/>
       <c r="H2" s="14"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14"/>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -6110,7 +4944,7 @@
       <c r="G3" s="14"/>
       <c r="H3" s="14"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14"/>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -6120,7 +4954,7 @@
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14"/>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -6130,7 +4964,7 @@
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14"/>
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
@@ -6140,7 +4974,7 @@
       <c r="G6" s="14"/>
       <c r="H6" s="14"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14"/>
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
@@ -6150,7 +4984,7 @@
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14"/>
       <c r="B8" s="14"/>
       <c r="C8" s="14"/>
@@ -6160,7 +4994,7 @@
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14"/>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
@@ -6170,7 +5004,7 @@
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14"/>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -6180,7 +5014,7 @@
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14"/>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
@@ -6190,7 +5024,7 @@
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14"/>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
@@ -6203,657 +5037,4 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00984AC6-2534-4DBE-B297-4A8ECA7B0506}">
-  <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B1" s="4">
-        <v>28250</v>
-      </c>
-      <c r="C1" s="14"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="4">
-        <v>28250</v>
-      </c>
-      <c r="C2" s="14"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="14"/>
-      <c r="B3" s="4">
-        <v>28250</v>
-      </c>
-      <c r="C3" s="14"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
-      <c r="B4" s="4">
-        <v>28250</v>
-      </c>
-      <c r="C4" s="14"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="14"/>
-      <c r="B5" s="4">
-        <v>28250</v>
-      </c>
-      <c r="C5" s="14"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
-      <c r="B6" s="4">
-        <v>28250</v>
-      </c>
-      <c r="C6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="B7" s="4">
-        <v>191030</v>
-      </c>
-      <c r="C7" s="14"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="B8" s="4">
-        <v>1316.66</v>
-      </c>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="B9" s="4">
-        <v>72406.5</v>
-      </c>
-      <c r="C9" s="14"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="B10" s="4">
-        <v>10520</v>
-      </c>
-      <c r="C10" s="14"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="B11" s="4">
-        <v>14000</v>
-      </c>
-      <c r="C11" s="14"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="B12" s="4">
-        <v>5000.01</v>
-      </c>
-      <c r="C12" s="14"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
-        <v>196</v>
-      </c>
-      <c r="B13" s="4">
-        <v>3116.3</v>
-      </c>
-      <c r="C13" s="14"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="B14" s="4">
-        <v>520.98</v>
-      </c>
-      <c r="C14" s="14"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="B15" s="4">
-        <v>7740</v>
-      </c>
-      <c r="C15" s="14"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
-        <v>200</v>
-      </c>
-      <c r="B16" s="4">
-        <v>4165</v>
-      </c>
-      <c r="C16" s="14"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B17" s="4">
-        <v>1770.31</v>
-      </c>
-      <c r="C17" s="14"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="14"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="14"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="14"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="14"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="14"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="14"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="14"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="14"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="14"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="14"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="14"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="14"/>
-      <c r="B27" s="4">
-        <f>SUM(B1:B26)</f>
-        <v>481085.75999999995</v>
-      </c>
-      <c r="C27" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2806F857-02AA-4E39-A9BD-4114EF397DE1}">
-  <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="27.5546875" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="B1" s="4">
-        <v>135085.5</v>
-      </c>
-      <c r="C1" s="14"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B2" s="4">
-        <v>56310</v>
-      </c>
-      <c r="C2" s="14"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="B3" s="4">
-        <v>12834.55</v>
-      </c>
-      <c r="C3" s="14"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="B4" s="4">
-        <v>6060</v>
-      </c>
-      <c r="C4" s="14"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="B5" s="4">
-        <v>457.93</v>
-      </c>
-      <c r="C5" s="14"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="B6" s="4">
-        <v>3850</v>
-      </c>
-      <c r="C6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="B7" s="4">
-        <v>10511.2</v>
-      </c>
-      <c r="C7" s="14"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="B8" s="4">
-        <v>2455.94</v>
-      </c>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="B9" s="4">
-        <v>1316.66</v>
-      </c>
-      <c r="C9" s="14"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="B10" s="4">
-        <v>2800</v>
-      </c>
-      <c r="C10" s="14"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="B11" s="4">
-        <v>4860</v>
-      </c>
-      <c r="C11" s="14"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="B12" s="4">
-        <v>2000</v>
-      </c>
-      <c r="C12" s="14"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B13" s="4">
-        <v>1331.49</v>
-      </c>
-      <c r="C13" s="14"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="14"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="14"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="14"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="14"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="14"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="14"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="14"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="14"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="14"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="14"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="14"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="14"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="14"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="14"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="14"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="14"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="14"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="14"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="14"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="14"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="14"/>
-      <c r="B28" s="4">
-        <f>SUM(B1:B27)</f>
-        <v>239873.27</v>
-      </c>
-      <c r="C28" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1D32F54-0432-4B6D-9D03-59ABDA4C02B1}">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22.5546875" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="B1" s="4">
-        <v>343854</v>
-      </c>
-      <c r="C1" s="14"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B2" s="4">
-        <v>72688.58</v>
-      </c>
-      <c r="C2" s="14"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B3" s="4">
-        <v>72688.58</v>
-      </c>
-      <c r="C3" s="14"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B4" s="4">
-        <v>72688.58</v>
-      </c>
-      <c r="C4" s="14"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B5" s="4">
-        <v>72688.58</v>
-      </c>
-      <c r="C5" s="14"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B6" s="4">
-        <v>72688.58</v>
-      </c>
-      <c r="C6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="B7" s="4">
-        <v>1316.66</v>
-      </c>
-      <c r="C7" s="14"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="B8" s="4">
-        <v>45371.78</v>
-      </c>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="B9" s="4">
-        <v>13250</v>
-      </c>
-      <c r="C9" s="14"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="4">
-        <v>998</v>
-      </c>
-      <c r="C10" s="14"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="B11" s="4">
-        <v>1069.21</v>
-      </c>
-      <c r="C11" s="14"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="B12" s="4">
-        <v>4800</v>
-      </c>
-      <c r="C12" s="14"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="B13" s="4">
-        <v>9900</v>
-      </c>
-      <c r="C13" s="14"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="B14" s="4">
-        <v>5000</v>
-      </c>
-      <c r="C14" s="14"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
-        <v>191</v>
-      </c>
-      <c r="B15" s="4">
-        <v>3764.82</v>
-      </c>
-      <c r="C15" s="14"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B16" s="4">
-        <v>2635.19</v>
-      </c>
-      <c r="C16" s="14"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="B17" s="4">
-        <v>20000</v>
-      </c>
-      <c r="C17" s="14"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="B18" s="4">
-        <v>998</v>
-      </c>
-      <c r="C18" s="14"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="14"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="14"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="14"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="14"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="14"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="14"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="14"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="14"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="14"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="14"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="14"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="14"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="14"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="14"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="14"/>
-      <c r="B29" s="4">
-        <f>SUM(B1:B28)</f>
-        <v>816400.55999999982</v>
-      </c>
-      <c r="C29" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>